<commit_message>
Inventario L10-M7: Recibido inicial Merlot (98/37/8/17); L9 y L34 en 0
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JXSZ5Q2QVHttNZRkf7MNkK
</commit_message>
<xml_diff>
--- a/Viñas Norte - Inventario L10-M7.xlsx
+++ b/Viñas Norte - Inventario L10-M7.xlsx
@@ -988,7 +988,9 @@
           <t>caja 1.4232 m² (2 pz)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
+      <c r="C5" s="5" t="n">
+        <v>98</v>
+      </c>
       <c r="D5" s="5">
         <f>SUMIF($B$12:$B$35,$A5,$C$12:$C$35)</f>
         <v/>
@@ -999,7 +1001,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>PENDIENTE LLENAR (aún hay piso)</t>
+          <t>Inicial Merlot (98/37/8/17) - resta lo usado</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1016,9 @@
           <t>caja 1.20 m² (5 pz)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
+      <c r="C6" s="5" t="n">
+        <v>37</v>
+      </c>
       <c r="D6" s="5">
         <f>SUMIF($B$12:$B$35,$A6,$C$12:$C$35)</f>
         <v/>
@@ -1036,7 +1040,9 @@
           <t>caja 1.35 m² (10 pz)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n"/>
+      <c r="C7" s="5" t="n">
+        <v>8</v>
+      </c>
       <c r="D7" s="5">
         <f>SUMIF($B$12:$B$35,$A7,$C$12:$C$35)</f>
         <v/>
@@ -1058,7 +1064,9 @@
           <t>pieza 0.30×0.60 m</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
+      <c r="C8" s="5" t="n">
+        <v>17</v>
+      </c>
       <c r="D8" s="5">
         <f>SUMIF($B$12:$B$35,$A8,$C$12:$C$35)</f>
         <v/>

</xml_diff>